<commit_message>
Fixed Line weights and P/B reference measurements for Er and Pr
</commit_message>
<xml_diff>
--- a/autoemx/data/Xray_lines/LineWeights_mod.xlsx
+++ b/autoemx/data/Xray_lines/LineWeights_mod.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Andrea_1/Desktop/Work/Codes/Repositories/AutoEMXSp/autoemx/data/Xray_lines/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A589FF6-9F09-C24D-9739-3A841E9FC5D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F36B401C-1CF7-1F49-863A-DEF5AD355699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40140" yWindow="2800" windowWidth="29920" windowHeight="18660" xr2:uid="{69DD2CB1-1C64-1C40-B86B-BA2360568088}"/>
+    <workbookView xWindow="39080" yWindow="9040" windowWidth="29920" windowHeight="18660" xr2:uid="{69DD2CB1-1C64-1C40-B86B-BA2360568088}"/>
   </bookViews>
   <sheets>
     <sheet name="LineWeights" sheetId="1" r:id="rId1"/>
@@ -14953,7 +14953,7 @@
         <v>0</v>
       </c>
       <c r="AF60" s="1">
-        <v>0.495</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="AG60" s="1">
         <v>3.9599999999999998E-4</v>
@@ -14995,7 +14995,7 @@
         <v>3.2699999999999999E-3</v>
       </c>
       <c r="AT60" s="1">
-        <v>0.111</v>
+        <v>9.2520000000000005E-2</v>
       </c>
       <c r="AU60" s="1">
         <v>0.1</v>
@@ -15028,10 +15028,10 @@
         <v>0</v>
       </c>
       <c r="BE60" s="1">
-        <v>4.3790000000000003E-2</v>
+        <v>0.1968</v>
       </c>
       <c r="BF60" s="1">
-        <v>0.28420000000000001</v>
+        <v>0.3049</v>
       </c>
       <c r="BG60" s="1">
         <v>0</v>
@@ -15058,7 +15058,7 @@
         <v>0</v>
       </c>
       <c r="BO60" s="1">
-        <v>0.4773</v>
+        <v>0.46189999999999998</v>
       </c>
       <c r="BP60" s="1">
         <v>0</v>
@@ -15070,7 +15070,7 @@
         <v>1.377</v>
       </c>
       <c r="BS60" s="1">
-        <v>0.14799999999999999</v>
+        <v>0.20130000000000001</v>
       </c>
       <c r="BT60" s="1">
         <v>7.6100000000000007E-5</v>
@@ -15082,7 +15082,7 @@
         <v>8.4500000000000006E-2</v>
       </c>
       <c r="BW60" s="1">
-        <v>1.716</v>
+        <v>3.714</v>
       </c>
       <c r="BX60">
         <v>0</v>
@@ -17007,14 +17007,14 @@
       <c r="Q69" s="1">
         <v>0</v>
       </c>
-      <c r="R69" s="1">
-        <v>8.7100000000000007E-3</v>
-      </c>
-      <c r="S69" s="1">
-        <v>7.7200000000000001E-4</v>
-      </c>
-      <c r="T69" s="1">
-        <v>4.8500000000000001E-2</v>
+      <c r="R69">
+        <v>6.9709999999999998E-3</v>
+      </c>
+      <c r="S69">
+        <v>2.2350000000000001E-4</v>
+      </c>
+      <c r="T69">
+        <v>3.5310000000000001E-2</v>
       </c>
       <c r="U69" s="1">
         <v>0</v>
@@ -17049,8 +17049,8 @@
       <c r="AE69" s="1">
         <v>0</v>
       </c>
-      <c r="AF69" s="1">
-        <v>0.50800000000000001</v>
+      <c r="AF69">
+        <v>0.41520000000000001</v>
       </c>
       <c r="AG69" s="1">
         <v>6.7500000000000004E-4</v>
@@ -17088,14 +17088,14 @@
       <c r="AR69" s="1">
         <v>0</v>
       </c>
-      <c r="AS69" s="1">
-        <v>1.06E-2</v>
-      </c>
-      <c r="AT69" s="1">
-        <v>0.105</v>
-      </c>
-      <c r="AU69" s="1">
-        <v>6.2799999999999995E-2</v>
+      <c r="AS69">
+        <v>3.0690000000000001E-3</v>
+      </c>
+      <c r="AT69">
+        <v>8.4029999999999994E-2</v>
+      </c>
+      <c r="AU69">
+        <v>5.1319999999999998E-2</v>
       </c>
       <c r="AV69" s="1">
         <v>0</v>
@@ -17127,8 +17127,8 @@
       <c r="BE69" s="1">
         <v>3.1600000000000003E-2</v>
       </c>
-      <c r="BF69" s="1">
-        <v>6.9900000000000004E-2</v>
+      <c r="BF69">
+        <v>7.5490000000000002E-2</v>
       </c>
       <c r="BG69" s="1">
         <v>0</v>
@@ -17154,8 +17154,8 @@
       <c r="BN69" s="1">
         <v>0</v>
       </c>
-      <c r="BO69" s="1">
-        <v>9.6299999999999997E-2</v>
+      <c r="BO69">
+        <v>0.16600000000000001</v>
       </c>
       <c r="BP69" s="1">
         <v>0</v>
@@ -17164,10 +17164,10 @@
         <v>5.4699999999999996E-4</v>
       </c>
       <c r="BR69" s="1">
-        <v>0.99099999999999999</v>
-      </c>
-      <c r="BS69" s="1">
-        <v>7.4800000000000005E-2</v>
+        <v>1.5680000000000001</v>
+      </c>
+      <c r="BS69">
+        <v>0.10970000000000001</v>
       </c>
       <c r="BT69" s="1">
         <v>1.85E-4</v>
@@ -17178,8 +17178,8 @@
       <c r="BV69" s="1">
         <v>1</v>
       </c>
-      <c r="BW69" s="1">
-        <v>0.45</v>
+      <c r="BW69">
+        <v>0.66020000000000001</v>
       </c>
       <c r="BX69">
         <v>0</v>

</xml_diff>